<commit_message>
fix(template): rename SKU to Артикул in orders import templates
</commit_message>
<xml_diff>
--- a/public/templates/orders-import-template.xlsx
+++ b/public/templates/orders-import-template.xlsx
@@ -1,28 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dvinskikh.sergey\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572BF8EF-DD0D-41B5-BD07-A55133EA293D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Заказы" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Заказы" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
-    <t>SKU</t>
+    <t>Номер заказа</t>
+  </si>
+  <si>
+    <t>Получатель</t>
+  </si>
+  <si>
+    <t>Телефон</t>
+  </si>
+  <si>
+    <t>Адрес</t>
+  </si>
+  <si>
+    <t>Комментарий</t>
+  </si>
+  <si>
+    <t>Артикул</t>
+  </si>
+  <si>
+    <t>Наименование</t>
+  </si>
+  <si>
+    <t>Количество</t>
+  </si>
+  <si>
+    <t>Внешний id</t>
   </si>
   <si>
     <t>10001</t>
@@ -55,6 +73,9 @@
     <t>Болт М10</t>
   </si>
   <si>
+    <t>ORD-10002</t>
+  </si>
+  <si>
     <t>10002</t>
   </si>
   <si>
@@ -76,47 +97,27 @@
     <t>Ремень 20мм</t>
   </si>
   <si>
-    <t>ORD-10002</t>
-  </si>
-  <si>
     <t>ORD-10003</t>
-  </si>
-  <si>
-    <t>Номер заказа</t>
-  </si>
-  <si>
-    <t>Получатель</t>
-  </si>
-  <si>
-    <t>Телефон</t>
-  </si>
-  <si>
-    <t>Адрес</t>
-  </si>
-  <si>
-    <t>Комментарий</t>
-  </si>
-  <si>
-    <t>Наименование</t>
-  </si>
-  <si>
-    <t>Количество</t>
-  </si>
-  <si>
-    <t>Внешний id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -181,22 +182,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -529,9 +530,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -542,127 +543,127 @@
     <col min="8" max="8" width="11.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1">
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H3" s="1">
         <v>6</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="H4" s="1">
         <v>2</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1216,60 +1217,57 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="I41:J41"/>
     <mergeCell ref="I42:J42"/>
     <mergeCell ref="I43:J43"/>
     <mergeCell ref="I44:J44"/>
     <mergeCell ref="I45:J45"/>
     <mergeCell ref="I46:J46"/>
     <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="F1 A4:H4 A2:G2 I2 A3:H3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>